<commit_message>
docs: clarify tenant import template guidance
</commit_message>
<xml_diff>
--- a/backend-api/resources/templates/tenant-import.xlsx
+++ b/backend-api/resources/templates/tenant-import.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Huong dan" sheetId="1" r:id="R82a90e378cf24184"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nguoi thue" sheetId="2" r:id="Rc55cd0c55fd343ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Huong dan" sheetId="1" r:id="Rb39028ee0b344883"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nguoi thue" sheetId="2" r:id="Rc79aca57053742ff"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,7 +18,7 @@
     <x:numFmt numFmtId="200" formatCode="@"/>
     <x:numFmt numFmtId="201" formatCode="dd/mm/yyyy"/>
   </x:numFmts>
-  <x:fonts count="4">
+  <x:fonts count="10">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -38,8 +38,44 @@
       <x:sz val="14"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF9A3412"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF1D4ED8"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFA16207"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF6D28D9"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFB91C1C"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFC2410C"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -51,8 +87,43 @@
         <x:fgColor rgb="FF1E293B"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4E5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1E293B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEFF6FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFEFCE8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF5F3FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFEF2F2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF7ED"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="1">
+  <x:borders count="7">
     <x:border>
       <x:left/>
       <x:right/>
@@ -60,11 +131,85 @@
       <x:bottom/>
       <x:diagonal/>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFF59E0B"/>
+      </x:left>
+      <x:right/>
+      <x:top style="thin">
+        <x:color rgb="FFF59E0B"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFF59E0B"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top style="thin">
+        <x:color rgb="FFF59E0B"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFF59E0B"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right style="thin">
+        <x:color rgb="FFF59E0B"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFF59E0B"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFF59E0B"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:left>
+      <x:right/>
+      <x:top style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="11">
+  <x:cellXfs count="55">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -78,6 +223,110 @@
     <x:xf numFmtId="201" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -315,96 +564,112 @@
       <x:c r="H2" t="str"/>
       <x:c r="I2" t="str"/>
     </x:row>
-    <x:row r="3" ht="25" customHeight="1">
-      <x:c r="A3" s="5" t="str">
-        <x:v>Chỉ nhập dữ liệu thật vào sheet Nguoi thue. Sheet này chỉ hướng dẫn và ví dụ, không được import.</x:v>
+    <x:row r="3" ht="36" customHeight="1">
+      <x:c r="A3" s="15" t="str">
+        <x:v>QUAN TRỌNG: Chỉ nhập dữ liệu vào sheet "Nguoi thue", từ dòng 2. Sheet "Huong dan" chỉ để xem hướng dẫn và ví dụ; dữ liệu điền tại đây sẽ không được import.</x:v>
       </x:c>
-      <x:c r="B3" s="5" t="str"/>
-      <x:c r="C3" s="5" t="str"/>
-      <x:c r="D3" s="5" t="str"/>
-      <x:c r="E3" s="5" t="str"/>
-      <x:c r="F3" s="5" t="str"/>
-      <x:c r="G3" s="5" t="str"/>
-      <x:c r="H3" s="5" t="str"/>
-      <x:c r="I3" s="5" t="str"/>
-    </x:row>
-    <x:row r="4" ht="25" customHeight="1">
-      <x:c r="A4" s="5" t="str">
-        <x:v>Chỉ Họ và tên bắt buộc. Giữ nguyên 6 header đầu; 3 cột cuối là tùy chọn.</x:v>
+      <x:c r="B3" s="16" t="str">
+        <x:v>QUAN TRỌNG: Chỉ nhập dữ liệu vào sheet "Nguoi thue", từ dòng 2. Sheet "Huong dan" chỉ để xem hướng dẫn và ví dụ; dữ liệu điền tại đây sẽ không được import.</x:v>
       </x:c>
-      <x:c r="B4" s="5" t="str"/>
-      <x:c r="C4" s="5" t="str"/>
-      <x:c r="D4" s="5" t="str"/>
-      <x:c r="E4" s="5" t="str"/>
-      <x:c r="F4" s="5" t="str"/>
-      <x:c r="G4" s="5" t="str"/>
-      <x:c r="H4" s="5" t="str"/>
-      <x:c r="I4" s="5" t="str"/>
-    </x:row>
-    <x:row r="5" ht="25" customHeight="1">
-      <x:c r="A5" s="5" t="str">
-        <x:v>Giới hạn: .xlsx, 5 MB, 1.000 người thuê. Mỗi dòng một hồ sơ.</x:v>
+      <x:c r="C3" s="16" t="str">
+        <x:v>QUAN TRỌNG: Chỉ nhập dữ liệu vào sheet "Nguoi thue", từ dòng 2. Sheet "Huong dan" chỉ để xem hướng dẫn và ví dụ; dữ liệu điền tại đây sẽ không được import.</x:v>
       </x:c>
-      <x:c r="B5" s="5" t="str"/>
-      <x:c r="C5" s="5" t="str"/>
-      <x:c r="D5" s="5" t="str"/>
-      <x:c r="E5" s="5" t="str"/>
-      <x:c r="F5" s="5" t="str"/>
-      <x:c r="G5" s="5" t="str"/>
-      <x:c r="H5" s="5" t="str"/>
-      <x:c r="I5" s="5" t="str"/>
-    </x:row>
-    <x:row r="6" ht="25" customHeight="1">
-      <x:c r="A6" s="5" t="str">
-        <x:v>Số điện thoại và CCCD/CMND: chọn định dạng Text TRƯỚC khi nhập để giữ số 0 đầu.</x:v>
+      <x:c r="D3" s="16" t="str">
+        <x:v>QUAN TRỌNG: Chỉ nhập dữ liệu vào sheet "Nguoi thue", từ dòng 2. Sheet "Huong dan" chỉ để xem hướng dẫn và ví dụ; dữ liệu điền tại đây sẽ không được import.</x:v>
       </x:c>
-      <x:c r="B6" s="5" t="str"/>
-      <x:c r="C6" s="5" t="str"/>
-      <x:c r="D6" s="5" t="str"/>
-      <x:c r="E6" s="5" t="str"/>
-      <x:c r="F6" s="5" t="str"/>
-      <x:c r="G6" s="5" t="str"/>
-      <x:c r="H6" s="5" t="str"/>
-      <x:c r="I6" s="5" t="str"/>
-    </x:row>
-    <x:row r="7" ht="25" customHeight="1">
-      <x:c r="A7" s="5" t="str">
-        <x:v>CCCD/CMND nếu có: đúng 9 hoặc 12 chữ số. SĐT: 9–15 chữ số, có thể có dấu + ở đầu.</x:v>
+      <x:c r="E3" s="16" t="str">
+        <x:v>QUAN TRỌNG: Chỉ nhập dữ liệu vào sheet "Nguoi thue", từ dòng 2. Sheet "Huong dan" chỉ để xem hướng dẫn và ví dụ; dữ liệu điền tại đây sẽ không được import.</x:v>
       </x:c>
-      <x:c r="B7" s="5" t="str"/>
-      <x:c r="C7" s="5" t="str"/>
-      <x:c r="D7" s="5" t="str"/>
-      <x:c r="E7" s="5" t="str"/>
-      <x:c r="F7" s="5" t="str"/>
-      <x:c r="G7" s="5" t="str"/>
-      <x:c r="H7" s="5" t="str"/>
-      <x:c r="I7" s="5" t="str"/>
-    </x:row>
-    <x:row r="8" ht="25" customHeight="1">
-      <x:c r="A8" s="5" t="str">
-        <x:v>Ngày sinh và Ngày cấp: DD/MM/YYYY, ví dụ 23/04/1995; hoặc ô ngày Excel. Không nhập ngày tương lai.</x:v>
+      <x:c r="F3" s="16" t="str">
+        <x:v>QUAN TRỌNG: Chỉ nhập dữ liệu vào sheet "Nguoi thue", từ dòng 2. Sheet "Huong dan" chỉ để xem hướng dẫn và ví dụ; dữ liệu điền tại đây sẽ không được import.</x:v>
       </x:c>
-      <x:c r="B8" s="5" t="str"/>
-      <x:c r="C8" s="5" t="str"/>
-      <x:c r="D8" s="5" t="str"/>
-      <x:c r="E8" s="5" t="str"/>
-      <x:c r="F8" s="5" t="str"/>
-      <x:c r="G8" s="5" t="str"/>
-      <x:c r="H8" s="5" t="str"/>
-      <x:c r="I8" s="5" t="str"/>
-    </x:row>
-    <x:row r="9" ht="25" customHeight="1">
-      <x:c r="A9" s="5" t="str">
-        <x:v>Giới tính: Nam, Nữ, Khác hoặc để trống. Không dùng công thức, macro hoặc liên kết ngoài.</x:v>
+      <x:c r="G3" s="16" t="str">
+        <x:v>QUAN TRỌNG: Chỉ nhập dữ liệu vào sheet "Nguoi thue", từ dòng 2. Sheet "Huong dan" chỉ để xem hướng dẫn và ví dụ; dữ liệu điền tại đây sẽ không được import.</x:v>
       </x:c>
-      <x:c r="B9" s="5" t="str"/>
-      <x:c r="C9" s="5" t="str"/>
-      <x:c r="D9" s="5" t="str"/>
-      <x:c r="E9" s="5" t="str"/>
-      <x:c r="F9" s="5" t="str"/>
-      <x:c r="G9" s="5" t="str"/>
-      <x:c r="H9" s="5" t="str"/>
-      <x:c r="I9" s="5" t="str"/>
+      <x:c r="H3" s="16" t="str">
+        <x:v>QUAN TRỌNG: Chỉ nhập dữ liệu vào sheet "Nguoi thue", từ dòng 2. Sheet "Huong dan" chỉ để xem hướng dẫn và ví dụ; dữ liệu điền tại đây sẽ không được import.</x:v>
+      </x:c>
+      <x:c r="I3" s="17" t="str">
+        <x:v>QUAN TRỌNG: Chỉ nhập dữ liệu vào sheet "Nguoi thue", từ dòng 2. Sheet "Huong dan" chỉ để xem hướng dẫn và ví dụ; dữ liệu điền tại đây sẽ không được import.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="24" customHeight="1">
+      <x:c r="A4" s="19" t="str">
+        <x:v>LƯU Ý ĐỂ IMPORT THÀNH CÔNG</x:v>
+      </x:c>
+      <x:c r="B4" s="19" t="str"/>
+      <x:c r="C4" s="19" t="str"/>
+      <x:c r="D4" s="19" t="str"/>
+      <x:c r="E4" s="19" t="str"/>
+      <x:c r="F4" s="19" t="str"/>
+      <x:c r="G4" s="19" t="str"/>
+      <x:c r="H4" s="19" t="str"/>
+      <x:c r="I4" s="19" t="str"/>
+    </x:row>
+    <x:row r="5" ht="30" customHeight="1">
+      <x:c r="A5" s="24" t="str">
+        <x:v>1. Header phải giữ nguyên tên. Có thể đổi thứ tự trong 9 cột A–I, nhưng không được thêm cột.</x:v>
+      </x:c>
+      <x:c r="B5" s="25" t="str"/>
+      <x:c r="C5" s="25" t="str"/>
+      <x:c r="D5" s="25" t="str"/>
+      <x:c r="E5" s="25" t="str"/>
+      <x:c r="F5" s="25" t="str"/>
+      <x:c r="G5" s="25" t="str"/>
+      <x:c r="H5" s="25" t="str"/>
+      <x:c r="I5" s="26" t="str"/>
+    </x:row>
+    <x:row r="6" ht="30" customHeight="1">
+      <x:c r="A6" s="31" t="str">
+        <x:v>2. SĐT và CCCD/CMND phải giữ kiểu Text để không mất số 0 đầu. Không đổi sang Number.</x:v>
+      </x:c>
+      <x:c r="B6" s="32" t="str"/>
+      <x:c r="C6" s="32" t="str"/>
+      <x:c r="D6" s="32" t="str"/>
+      <x:c r="E6" s="32" t="str"/>
+      <x:c r="F6" s="32" t="str"/>
+      <x:c r="G6" s="32" t="str"/>
+      <x:c r="H6" s="32" t="str"/>
+      <x:c r="I6" s="33" t="str"/>
+    </x:row>
+    <x:row r="7" ht="30" customHeight="1">
+      <x:c r="A7" s="38" t="str">
+        <x:v>3. Ngày sinh/Ngày cấp dùng ô ngày Excel hoặc text DD/MM/YYYY. Không nhập text YYYY-MM-DD.</x:v>
+      </x:c>
+      <x:c r="B7" s="39" t="str"/>
+      <x:c r="C7" s="39" t="str"/>
+      <x:c r="D7" s="39" t="str"/>
+      <x:c r="E7" s="39" t="str"/>
+      <x:c r="F7" s="39" t="str"/>
+      <x:c r="G7" s="39" t="str"/>
+      <x:c r="H7" s="39" t="str"/>
+      <x:c r="I7" s="40" t="str"/>
+    </x:row>
+    <x:row r="8" ht="24" customHeight="1">
+      <x:c r="A8" s="45" t="str">
+        <x:v>4. Không dùng công thức trong ô dữ liệu.</x:v>
+      </x:c>
+      <x:c r="B8" s="46" t="str"/>
+      <x:c r="C8" s="46" t="str"/>
+      <x:c r="D8" s="46" t="str"/>
+      <x:c r="E8" s="46" t="str"/>
+      <x:c r="F8" s="46" t="str"/>
+      <x:c r="G8" s="46" t="str"/>
+      <x:c r="H8" s="46" t="str"/>
+      <x:c r="I8" s="47" t="str"/>
+    </x:row>
+    <x:row r="9" ht="30" customHeight="1">
+      <x:c r="A9" s="52" t="str">
+        <x:v>5. File mẫu có 2 sheet: chỉ nhập tại Nguoi thue. Không đổi tên sheet này hoặc điền dữ liệu ở Huong dan.</x:v>
+      </x:c>
+      <x:c r="B9" s="53" t="str"/>
+      <x:c r="C9" s="53" t="str"/>
+      <x:c r="D9" s="53" t="str"/>
+      <x:c r="E9" s="53" t="str"/>
+      <x:c r="F9" s="53" t="str"/>
+      <x:c r="G9" s="53" t="str"/>
+      <x:c r="H9" s="53" t="str"/>
+      <x:c r="I9" s="54" t="str"/>
     </x:row>
     <x:row r="10" ht="25" customHeight="1">
       <x:c r="A10" s="5" t="str">
@@ -538,6 +803,15 @@
       <x:c r="I16" s="5" t="str"/>
     </x:row>
   </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A3:I3"/>
+    <x:mergeCell ref="A4:I4"/>
+    <x:mergeCell ref="A5:I5"/>
+    <x:mergeCell ref="A6:I6"/>
+    <x:mergeCell ref="A7:I7"/>
+    <x:mergeCell ref="A8:I8"/>
+    <x:mergeCell ref="A9:I9"/>
+  </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>

</xml_diff>